<commit_message>
Tambah data bumil: MIANA (NIK 3209376507960002)
</commit_message>
<xml_diff>
--- a/Penerima Manfaat (1).xlsx
+++ b/Penerima Manfaat (1).xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>NISN/NIK</t>
   </si>
@@ -221,6 +221,15 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>3209376507960002</t>
+  </si>
+  <si>
+    <t>MIANA</t>
+  </si>
+  <si>
+    <t>25-07-1996</t>
   </si>
 </sst>
 </file>
@@ -541,7 +550,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -620,6 +629,29 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4">
+        <v>64</v>
+      </c>
+      <c r="E4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>